<commit_message>
feat(catalog): "bowl"-Tag gilt jetzt auch für Salate
30 Salate haben den Tag bekommen, damit sind es 50 statt 20 (19 Bowls,
31 Salate).

Maßstab ist das Kopf-Nomen: Das Gericht muss eine Bowl oder ein Salat
SEIN. Vier Gerichte haben "Salat" im Namen, ohne einer zu sein — dort
ist er Beilage oder Zutat, und sie bleiben ungetaggt:
  - LC Wrap Räucherlachs + Cottage + Salat        (Wrap)
  - LC Wrap Salat + Walnüsse + Gurke + Paprika    (Wrap)
  - Lachs vom Grill mit Apfel-Gurken-Salat        (Beilagensalat)
  - Gegrillter Lachs mit Salat, Quinoa, Blutorangen (Beilagensalat)

"Lachs auf Quinoasalat" ist dagegen getaggt: Der Salat ist dort die
Basis des Gerichts, nicht die Beilage.

autotags() im Konverter bleibt unverändert — die Funktion zerlegt nur
den Namen in Suchtokens und hat keine Semantik; die Tags in Spalte H
sind kuratiert.

Katalog 7 → 8, Regel im README dokumentiert.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/dishes 2.0.xlsx
+++ b/data/dishes 2.0.xlsx
@@ -759,7 +759,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>süß, kalt, meal prep, cheat</t>
+          <t>bowl, süß, kalt, meal prep, cheat</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>leicht verdaulich, kalt, meal prep, vegetarisch</t>
+          <t>bowl, leicht verdaulich, kalt, meal prep, vegetarisch</t>
         </is>
       </c>
       <c r="I12" s="12" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go</t>
+          <t>bowl, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go</t>
+          <t>bowl, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I14" s="12" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, vegetarisch, cheat</t>
+          <t>bowl, kalt, meal prep, vegetarisch, cheat</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep</t>
+          <t>bowl, kalt, meal prep</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go</t>
+          <t>bowl, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr">
@@ -6193,7 +6193,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>süß, kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, süß, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go</t>
+          <t>bowl, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>kalt, vegetarisch, cheat</t>
+          <t>bowl, kalt, vegetarisch, cheat</t>
         </is>
       </c>
       <c r="I141" s="2" t="inlineStr">
@@ -8741,7 +8741,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I173" s="13" t="inlineStr">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>leicht verdaulich, kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, leicht verdaulich, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="J175" s="7" t="n"/>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>leicht verdaulich, kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, leicht verdaulich, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="J176" s="7" t="n"/>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>leicht verdaulich, kalt, meal prep, to go</t>
+          <t>bowl, leicht verdaulich, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I221" s="13" t="inlineStr">
@@ -11621,7 +11621,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>kalt</t>
+          <t>bowl, kalt</t>
         </is>
       </c>
       <c r="I222" s="13" t="inlineStr">
@@ -11684,7 +11684,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go</t>
+          <t>bowl, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I223" s="13" t="inlineStr">
@@ -11754,7 +11754,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>süß, kalt, meal prep, vegetarisch</t>
+          <t>bowl, süß, kalt, meal prep, vegetarisch</t>
         </is>
       </c>
       <c r="I224" s="13" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>warm, meal prep, to go, vegetarisch</t>
+          <t>bowl, warm, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I225" s="13" t="inlineStr">
@@ -11879,7 +11879,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>leicht verdaulich, kalt, meal prep, to go</t>
+          <t>bowl, leicht verdaulich, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I226" s="13" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I227" s="13" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I228" s="13" t="inlineStr">
@@ -12060,7 +12060,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I229" s="13" t="inlineStr">
@@ -12121,7 +12121,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>leicht verdaulich, kalt, vegetarisch</t>
+          <t>bowl, leicht verdaulich, kalt, vegetarisch</t>
         </is>
       </c>
       <c r="I230" s="13" t="inlineStr">
@@ -12181,7 +12181,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go</t>
+          <t>bowl, kalt, meal prep, to go</t>
         </is>
       </c>
       <c r="I231" s="13" t="inlineStr">
@@ -12240,7 +12240,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>kalt</t>
+          <t>bowl, kalt</t>
         </is>
       </c>
       <c r="I232" s="13" t="inlineStr">
@@ -13102,7 +13102,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I246" s="13" t="inlineStr">
@@ -13450,7 +13450,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>kalt, meal prep, to go, vegetarisch</t>
+          <t>bowl, kalt, meal prep, to go, vegetarisch</t>
         </is>
       </c>
       <c r="I252" s="13" t="inlineStr">

</xml_diff>